<commit_message>
Implement inline JS mobile menu toggle handler
</commit_message>
<xml_diff>
--- a/Movie Archive Inputs.xlsx
+++ b/Movie Archive Inputs.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Creative\Podcasts\Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD4D2A1-218C-4982-BCEA-37AB0A8980C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391265F8-4D4C-4529-8EB0-F7C737A9E767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Movie Ratings" sheetId="1" r:id="rId1"/>
     <sheet name="Transcripts" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Movie Ratings'!$A$1:$F$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Movie Ratings'!$A$1:$F$38</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="152">
   <si>
     <t>12 Angry Men</t>
   </si>
@@ -7094,6 +7094,12 @@
 Darius: You know, I the Weaponizing the power of male *****. Right. You know, I, it's like I've seen men willing to walk across hot coals barefoot to get, you know, to *** ****. It's so, and so that, and you know, they're pretty women, so they're harmless. And then the cops, how long did the cops hang up on people calling to try to report them? Right. it's just the entire premise of this was them believing that no one would take male victims seriously. Yeah. Yes.
 Jordan: Do you? Okay, so it might be for actor. I don't know. So there's a portion of interview where she, you can almost hear Constance Wu's character like bargaining almost like an addict where she's like, no, you have to understand like, We didn't think we were doing anything wrong. We're like, you have to understand these were guys who, would have, co</t>
   </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=VzrFB2-GMt0&amp;t=2s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pVgVo-IvEVQ&amp;t=963s</t>
+  </si>
 </sst>
 </file>
 
@@ -7166,7 +7172,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -7191,6 +7197,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -7207,10 +7214,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7658,7 +7661,7 @@
         <v>115</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
@@ -7772,8 +7775,8 @@
       <c r="E12" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="F12" t="s">
-        <v>40</v>
+      <c r="F12" s="10" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="391.5" x14ac:dyDescent="0.25">
@@ -8289,7 +8292,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F38" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{8E5B87CC-F717-4172-93E2-C446A611ADD5}"/>
   </hyperlinks>

</xml_diff>

<commit_message>
Update site layout, host hierarchy, and archives
</commit_message>
<xml_diff>
--- a/Movie Archive Inputs.xlsx
+++ b/Movie Archive Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Creative\Podcasts\Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1EDCBC4-A91B-449B-8618-89F067AAE858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB789B41-965D-47B7-B68C-03AA97336FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Movie Ratings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="159">
   <si>
     <t>12 Angry Men</t>
   </si>
@@ -7617,6 +7617,9 @@
 Jordan: Okay.
 Darius: You know, like even if you're like, Even if you're in the mall, don't try not to break character. Don't break character in interviews because like yo</t>
   </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=PO9gS2D0P7o&amp;t=1s</t>
+  </si>
 </sst>
 </file>
 
@@ -7730,10 +7733,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8550,6 +8549,9 @@
       <c r="E25" s="9" t="s">
         <v>133</v>
       </c>
+      <c r="F25" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">

</xml_diff>